<commit_message>
Align employee bulk imports with table updates, verify excel templates columns, add storage asset helper in templates, and update tests
</commit_message>
<xml_diff>
--- a/public/assets/excel/employee_salary_breakdown.xlsx
+++ b/public/assets/excel/employee_salary_breakdown.xlsx
@@ -1,90 +1,94 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24326"/>
-  <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo LOQ\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{695A670F-EEE5-4E7D-859A-8B8EABC14600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
   <si>
     <t>Employee_id</t>
   </si>
   <si>
+    <t>APP000001</t>
+  </si>
+  <si>
+    <t>APP000002</t>
+  </si>
+  <si>
+    <t>APP000003</t>
+  </si>
+  <si>
+    <t>APP000004</t>
+  </si>
+  <si>
+    <t>APP000005</t>
+  </si>
+  <si>
+    <t>BDT</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>Gross_salary</t>
+  </si>
+  <si>
+    <t>Other_earnings</t>
+  </si>
+  <si>
+    <t>Medical_allowance</t>
+  </si>
+  <si>
+    <t>Food_allowance</t>
+  </si>
+  <si>
+    <t>Transport_allowance</t>
+  </si>
+  <si>
+    <t>House_allowance</t>
+  </si>
+  <si>
     <t>Basic_salary</t>
   </si>
   <si>
-    <t>House_allowance</t>
-  </si>
-  <si>
-    <t>Transport_allowance</t>
-  </si>
-  <si>
-    <t>Food_allowance</t>
-  </si>
-  <si>
-    <t>Medical_allowance</t>
-  </si>
-  <si>
-    <t>Other_earnings</t>
-  </si>
-  <si>
-    <t>Gross_salary</t>
-  </si>
-  <si>
-    <t>Currency</t>
-  </si>
-  <si>
-    <t>BDT</t>
-  </si>
-  <si>
-    <t>APP000001</t>
-  </si>
-  <si>
-    <t>APP000002</t>
-  </si>
-  <si>
-    <t>APP000003</t>
-  </si>
-  <si>
-    <t>APP000004</t>
-  </si>
-  <si>
-    <t>APP000005</t>
+    <t>Pay Scale</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -106,16 +110,16 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -124,24 +128,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -188,7 +184,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -240,7 +236,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -465,198 +461,220 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5546875" customWidth="true" style="0"/>
+    <col min="3" max="3" width="10.88671875" customWidth="true" style="0"/>
+    <col min="4" max="4" width="15.5546875" customWidth="true" style="0"/>
+    <col min="5" max="5" width="18.6640625" customWidth="true" style="0"/>
+    <col min="6" max="6" width="14.44140625" customWidth="true" style="0"/>
+    <col min="7" max="7" width="16.77734375" customWidth="true" style="0"/>
+    <col min="8" max="8" width="13.88671875" customWidth="true" style="0"/>
+    <col min="9" max="9" width="11.44140625" customWidth="true" style="0"/>
+    <col min="10" max="10" width="8.21875" customWidth="true" style="0"/>
+    <col min="11" max="11" width="12.88671875" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
+      <c r="B1" t="s">
+        <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1"/>
+      <c r="J1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="1"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
         <v>50000</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>10000</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>5000</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>2000</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>3000</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>1000</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>83000</v>
       </c>
-      <c r="I2" t="s">
-        <v>9</v>
-      </c>
+      <c r="J2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
         <v>55000</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>12000</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>6000</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>2500</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>3500</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>1500</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>97000</v>
       </c>
-      <c r="I3" t="s">
-        <v>9</v>
-      </c>
+      <c r="J3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K3"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
         <v>60000</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>15000</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>7000</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>3000</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>4000</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>2000</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>113000</v>
       </c>
-      <c r="I4" t="s">
-        <v>9</v>
-      </c>
+      <c r="J4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K4"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
         <v>45000</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>8000</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>4000</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>1500</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>2500</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>1000</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>69500</v>
       </c>
-      <c r="I5" t="s">
-        <v>9</v>
-      </c>
+      <c r="J5" t="s">
+        <v>6</v>
+      </c>
+      <c r="K5"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
         <v>52000</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>10000</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>5000</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>2000</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>3000</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>1200</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>83200</v>
       </c>
-      <c r="I6" t="s">
-        <v>9</v>
-      </c>
+      <c r="J6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K6"/>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>